<commit_message>
chore(qa): regenerate Excel report and sync VC-012/014/023/024/029 to Jira
Transitioned all five to Done with a fix-summary comment on each issue.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-12 03:44 UTC</t>
+          <t>Generated 2026-09-12 04:37 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -12758,7 +12758,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -12861,7 +12861,7 @@
       </c>
       <c r="AA13" s="5" t="inlineStr">
         <is>
-          <t>Could not be observed in this run: no Android &lt;= 12 device or AVD is available on this machine. Needs a real 3 GB Android 10 device to close.</t>
+          <t>FIX: refreshPermission() (pushService.ts) trusted hasNotificationPermission() alone, which on Android &lt;33 has no runtime dialog and unconditionally answers true regardless of the app-level or channel-level notification toggle the user can flip from system Settings. Combined it with the same native areMessageNotificationsBlocked() check the push blocker banner already used (getPushBlocker()), via a new pure decision function notificationsGranted(permitted, blocked) in pushState.ts, so permission now genuinely means the OS will show something on every API level before isPushAvailable lets the SyncEngine drop its background socket. No native code changed — reused the existing native primitive. Verified: full jest suite 456/456 pass (452 + 4 new), tsc --noEmit clean, eslint 0 errors on touched files. Could not be observed on a real Android &lt;=12 device (none available on this machine) — the fix is verified at the unit-test level against the exact documented defect (permitted=true, blocked=true -&gt; denied), not end-to-end on hardware.</t>
         </is>
       </c>
     </row>
@@ -13015,7 +13015,11 @@
           <t>VC-17</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>authStore.test.ts: VC-014</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Rotating-refresh replay is structurally inevitable on a lost response, and the family revoke is then silently swallowed</t>
@@ -13033,7 +13037,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -13137,7 +13141,7 @@
       </c>
       <c r="AA15" s="5" t="inlineStr">
         <is>
-          <t>No automated test currently exercises the client-side claim (device re-login after a family revoke swallows the signal). VC-AUTH-024 was removed from testIds: it verifies the BACKEND's revoke-on-reuse behaviour (confirmed working since the first run) but says nothing about the client. Needs an RN-level test or a manual repro to close.</t>
+          <t>FIX (investigated against the real backend source at D:Velchat, read-only): confirmed a refresh-reuse family revoke and a plain invalid/expired refresh both return an identical 401 UNAUTHORIZED with no distinguishing code, and confirmed device-key login is architecturally INDEPENDENT of the refresh-token family (revokeFamily only touches refresh_tokens; the devices table has no family_id) - so a device that still holds its private key can always mint a fresh session, and the client cannot and need not distinguish reuse-triggered revokes from ordinary rejections. Two real defects fixed: (1) clearSession() was deleting KVKeys.deviceId, which meant NEITHER the existing cold-start silent-relogin (useAuthBootstrap) NOR any warm recovery could ever actually reach /auth/challenge after a forced expiry, despite the code comments claiming this already worked - moved the explicit deviceId wipe into signOut() only, so a real logout is unchanged but a forced expiry now keeps it, same as the device key. (2) added attemptSilentRelogin() (authStore.ts), invoked from sessionExpired() itself, so a lost-refresh-response false-positive family revoke recovers IMMEDIATELY while the app is warm instead of only on the next cold start, turning a network hiccup back into nothing instead of stranding the user on the sign-in screen. Did not attempt to prevent the reuse-detection race itself (structurally requires a backend idempotency mechanism - out of scope, frontend-only per current instruction). Verified: full jest suite 481/481 pass, tsc --noEmit clean, eslint 0 errors. No RN-level test existed before; added 4 new tests (authStore.test.ts) covering the success, no-device-key, device-revoked and sessionExpired-wiring paths - the second and third caught the deviceId-wipe bug during RED before the fix was written.</t>
         </is>
       </c>
     </row>
@@ -14281,7 +14285,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -14381,7 +14385,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="AA24" s="5" t="inlineStr"/>
+      <c r="AA24" s="5" t="inlineStr">
+        <is>
+          <t>FIX: classifySendFailure() grouped auth with client, treating a post-refresh-failure 401/403 as if THIS message were rejected (permanent:true, pauseDrain:false) — one transient auth hiccup then permanently failed every other queued message as the drain kept walking into the same 401. auth is a SESSION problem, not a message problem (client.ts already treats a refresh that cannot reach the server as retryable, leaving the session valid). Added a dedicated auth case returning {permanent:false, pauseDrain:true, cooldownMs:0}, matching the network/timeout/server treatment, so the drain pauses instead of destroying the queue and resumes once the session recovers. Split the existing it.each(['client','auth']) test (which encoded the old, wrong grouping) into client-only plus a new dedicated describe block for auth. Verified: full jest suite 452/452 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -14396,7 +14404,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-205</t>
+          <t>schema.test.ts: VC-024</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -14416,7 +14424,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -14517,7 +14525,7 @@
       </c>
       <c r="AA25" s="5" t="inlineStr">
         <is>
-          <t>migrations.test.ts tests the declaration, not the effect.</t>
+          <t>FIX: added an unsafeSql hook to schema.ts (appSchema) — WatermelonDB's own supported extension point, confirmed by reading adapters/sqlite/encodeSchema/index.js (encodeSchema calls unsafeSql(sql, "setup") for a fresh install) — that appends the same five composite CREATE INDEX statements the v3 migration already applies on an upgrade. Extracted the five statements into a new shared compositeIndexes.ts so migrations.ts and schema.ts can never drift apart, and migrations.ts now maps over that same array instead of repeating the SQL inline. Verified: full jest suite 481/481 pass (3 new tests in schema.test.ts assert the hook exists, appends every composite index on kind:"setup", and leaves other DDL kinds untouched), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
@@ -15096,7 +15104,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -15197,7 +15205,7 @@
       </c>
       <c r="AA30" s="5" t="inlineStr">
         <is>
-          <t>Two existing tests cover code that cannot run in production.</t>
+          <t>FIX: removed the dead attempt-count exhaustion path (MAX_SEND_ATTEMPTS/nextOutboxRetry in syncLogic.ts) that markFailed() fell back to only when permanent was omitted — a fallback no real call site ever triggered (SyncEngine.ts always passes a classified boolean from classifySendFailure()). This mechanism contradicted the documented WhatsApp-style policy (sendFailurePolicy.ts: reachability failures retry forever, never auto-fail by attempt count) and had no basis in the HLD/LLD spec (§L6 outbox semantics: classification-based retryable-vs-permanent only, no attempt cap). Made markFailed()'s permanent parameter required (compiler now prevents the dead path from ever coming back), updated the one test that accidentally relied on the old default (realtime-hardening.test.ts) to pass permanent explicitly, removed the 4 tests for the deleted dead function, and added a new regression test proving a retryable cause stays queued past a high attempt count. Verified: full jest suite 452/452 pass (455 - 4 removed + 1 added), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
@@ -17148,7 +17156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -17334,7 +17342,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -17345,7 +17353,7 @@
         </is>
       </c>
       <c r="B19" s="22" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C19" s="23" t="inlineStr"/>
     </row>
@@ -17404,7 +17412,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>23 open P0/P1 defect(s) block the build.</t>
+          <t>20 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -17556,7 +17564,7 @@
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
         <is>
-          <t>VC-012</t>
+          <t>VC-016</t>
         </is>
       </c>
       <c r="B37" s="22" t="inlineStr">
@@ -17566,14 +17574,14 @@
       </c>
       <c r="C37" s="23" t="inlineStr">
         <is>
-          <t>Android &lt;= 12 reports notifications as granted even when disabled, so the sync engine drops its background socket</t>
+          <t>MMKV's encryption key is a hardcoded bundle constant, and the Ed25519 device private key is stored inside it</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="21" t="inlineStr">
         <is>
-          <t>VC-014</t>
+          <t>VC-017</t>
         </is>
       </c>
       <c r="B38" s="22" t="inlineStr">
@@ -17583,31 +17591,31 @@
       </c>
       <c r="C38" s="23" t="inlineStr">
         <is>
-          <t>Rotating-refresh replay is structurally inevitable on a lost response, and the family revoke is then silently swallowed</t>
+          <t>Message plaintext and the user's own typed replies persist in plaintext SharedPreferences</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="inlineStr">
         <is>
-          <t>VC-016</t>
+          <t>VC-018</t>
         </is>
       </c>
       <c r="B39" s="22" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C39" s="23" t="inlineStr">
         <is>
-          <t>MMKV's encryption key is a hardcoded bundle constant, and the Ed25519 device private key is stored inside it</t>
+          <t>No certificate pinning anywhere, in JS or native</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>VC-017</t>
+          <t>VC-025</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
@@ -17617,14 +17625,14 @@
       </c>
       <c r="C40" s="23" t="inlineStr">
         <is>
-          <t>Message plaintext and the user's own typed replies persist in plaintext SharedPreferences</t>
+          <t>reassertReceipts() on every connect emits an unbounded burst the gateway silently drops</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>VC-018</t>
+          <t>VC-028</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
@@ -17634,14 +17642,14 @@
       </c>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>No certificate pinning anywhere, in JS or native</t>
+          <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
-          <t>VC-023</t>
+          <t>VC-030</t>
         </is>
       </c>
       <c r="B42" s="22" t="inlineStr">
@@ -17651,14 +17659,14 @@
       </c>
       <c r="C42" s="23" t="inlineStr">
         <is>
-          <t>One 401 on send turns the entire outbox into permanently failed messages</t>
+          <t>Message window sorts by created_at, not seq — a device clock ahead of the server permanently mis-orders own messages</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
         <is>
-          <t>VC-025</t>
+          <t>VC-032</t>
         </is>
       </c>
       <c r="B43" s="22" t="inlineStr">
@@ -17668,14 +17676,14 @@
       </c>
       <c r="C43" s="23" t="inlineStr">
         <is>
-          <t>reassertReceipts() on every connect emits an unbounded burst the gateway silently drops</t>
+          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
         <is>
-          <t>VC-028</t>
+          <t>VC-033</t>
         </is>
       </c>
       <c r="B44" s="22" t="inlineStr">
@@ -17685,31 +17693,31 @@
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>No event_id dedup anywhere — the documented at-least-once guard does not exist</t>
+          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="inlineStr">
         <is>
-          <t>VC-030</t>
+          <t>VC-039</t>
         </is>
       </c>
       <c r="B45" s="22" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Message window sorts by created_at, not seq — a device clock ahead of the server permanently mis-orders own messages</t>
+          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="inlineStr">
         <is>
-          <t>VC-032</t>
+          <t>VC-040</t>
         </is>
       </c>
       <c r="B46" s="22" t="inlineStr">
@@ -17719,14 +17727,14 @@
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>No duplicate-notification suppression, though the monotonic watermark to do it already exists</t>
+          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="21" t="inlineStr">
         <is>
-          <t>VC-033</t>
+          <t>VC-041</t>
         </is>
       </c>
       <c r="B47" s="22" t="inlineStr">
@@ -17736,73 +17744,22 @@
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>Native pending-event queue is a lock-free read-modify-write that can wipe a reply enqueued mid-drain</t>
+          <t>POST /chat/messages accepts a conversationId that does not exist</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
         <is>
-          <t>VC-039</t>
+          <t>VC-043</t>
         </is>
       </c>
       <c r="B48" s="22" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
-        <is>
-          <t>Any authenticated user can READ and WRITE any conversation — no authorization on the chat routes, and conversation ids are derivable offline</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="21" t="inlineStr">
-        <is>
-          <t>VC-040</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="inlineStr">
-        <is>
-          <t>A push endpoint can be registered against another account's userId, redirecting their push wake-ups</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
-        <is>
-          <t>VC-041</t>
-        </is>
-      </c>
-      <c r="B50" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C50" s="23" t="inlineStr">
-        <is>
-          <t>POST /chat/messages accepts a conversationId that does not exist</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="21" t="inlineStr">
-        <is>
-          <t>VC-043</t>
-        </is>
-      </c>
-      <c r="B51" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C51" s="23" t="inlineStr">
         <is>
           <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
         </is>
@@ -17957,7 +17914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -18091,12 +18048,12 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>VC-013</t>
+          <t>VC-012</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>clearSession() is not a session teardown — the previous account's chat DB, profile and contacts survive into the next sign-in</t>
+          <t>Android &lt;= 12 reports notifications as granted even when disabled, so the sync engine drops its background socket</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -18111,7 +18068,7 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-104</t>
+          <t>VC-UNIT-103</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
@@ -18122,24 +18079,24 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>FIX: sessionExpired() now runs the same purgeAccountData() as signOut() (extracted, shared), minus clearDeviceKey() (a transient expiry must still allow a later silent relogin) and the network logout call (pointless — the session is already rejected). The next sign-in on this device, even under a different phone number, no longer inherits the previous account chat DB, profile, contacts or receipts. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: refreshPermission() (pushService.ts) trusted hasNotificationPermission() alone, which on Android &lt;33 has no runtime dialog and unconditionally answers true regardless of the app-level or channel-level notification toggle the user can flip from system Settings. Combined it with the same native areMessageNotificationsBlocked() check the push blocker banner already used (getPushBlocker()), via a new pure decision function notificationsGranted(permitted, blocked) in pushState.ts, so permission now genuinely means the OS will show something on every API level before isPushAvailable lets the SyncEngine drop its background socket. No native code changed — reused the existing native primitive. Verified: full jest suite 456/456 pass (452 + 4 new), tsc --noEmit clean, eslint 0 errors on touched files. Could not be observed on a real Android &lt;=12 device (none available on this machine) — the fix is verified at the unit-test level against the exact documented defect (permitted=true, blocked=true -&gt; denied), not end-to-end on hardware.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>VC-015</t>
+          <t>VC-013</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>The cnfJkt DPoP binding is dead code — the refresh token is bound to nothing</t>
+          <t>clearSession() is not a session teardown — the previous account's chat DB, profile and contacts survive into the next sign-in</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -18149,7 +18106,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-106</t>
+          <t>VC-UNIT-104</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
@@ -18160,24 +18117,24 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>FIX: Added cnfJktThumbprint() (deviceKey.ts) — a real RFC 7638 JWK thumbprint (RFC 8037 OKP encoding) over the device Ed25519 public key. doRefresh() now computes it fresh on every refresh instead of round-tripping through an MMKV key nothing ever wrote a real value into. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: sessionExpired() now runs the same purgeAccountData() as signOut() (extracted, shared), minus clearDeviceKey() (a transient expiry must still allow a later silent relogin) and the network logout call (pointless — the session is already rejected). The next sign-in on this device, even under a different phone number, no longer inherits the previous account chat DB, profile, contacts or receipts. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>VC-020</t>
+          <t>VC-014</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Concurrent applyServerMessages duplicates every row in the overlap, and can lose a whole batch on a conversation PK clash</t>
+          <t>Rotating-refresh replay is structurally inevitable on a lost response, and the family revoke is then silently swallowed</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -18187,7 +18144,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-201</t>
+          <t>authStore.test.ts: VC-014</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
@@ -18198,24 +18155,24 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>VC-001 makes this far more likely to be hit in practice, because seq gaps are constant. FIX: The three lookup queries in applyServerMessages moved inside db.write(), read before any prepareCreate/prepareUpdate call — closes the race without violating the prepare-then-batch-synchronously constraint. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX (investigated against the real backend source at D:Velchat, read-only): confirmed a refresh-reuse family revoke and a plain invalid/expired refresh both return an identical 401 UNAUTHORIZED with no distinguishing code, and confirmed device-key login is architecturally INDEPENDENT of the refresh-token family (revokeFamily only touches refresh_tokens; the devices table has no family_id) - so a device that still holds its private key can always mint a fresh session, and the client cannot and need not distinguish reuse-triggered revokes from ordinary rejections. Two real defects fixed: (1) clearSession() was deleting KVKeys.deviceId, which meant NEITHER the existing cold-start silent-relogin (useAuthBootstrap) NOR any warm recovery could ever actually reach /auth/challenge after a forced expiry, despite the code comments claiming this already worked - moved the explicit deviceId wipe into signOut() only, so a real logout is unchanged but a forced expiry now keeps it, same as the device key. (2) added attemptSilentRelogin() (authStore.ts), invoked from sessionExpired() itself, so a lost-refresh-response false-positive family revoke recovers IMMEDIATELY while the app is warm instead of only on the next cold start, turning a network hiccup back into nothing instead of stranding the user on the sign-in screen. Did not attempt to prevent the reuse-detection race itself (structurally requires a backend idempotency mechanism - out of scope, frontend-only per current instruction). Verified: full jest suite 481/481 pass, tsc --noEmit clean, eslint 0 errors. No RN-level test existed before; added 4 new tests (authStore.test.ts) covering the success, no-device-key, device-revoked and sessionExpired-wiring paths - the second and third caught the deviceId-wipe bug during RED before the fix was written.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>VC-021</t>
+          <t>VC-015</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>applyReceipt is a non-atomic read-modify-write, so blue ticks can regress to grey</t>
+          <t>The cnfJkt DPoP binding is dead code — the refresh token is bound to nothing</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -18225,7 +18182,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-202</t>
+          <t>VC-UNIT-106</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
@@ -18236,24 +18193,24 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Every existing receipt test applies receipts sequentially, which is exactly why they all pass. FIX: applyReceipt now re-fetches the rows to update from inside db.write() (same pattern as VC-020) instead of before it, so the monotonic check is atomic with the write. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: Added cnfJktThumbprint() (deviceKey.ts) — a real RFC 7638 JWK thumbprint (RFC 8037 OKP encoding) over the device Ed25519 public key. doRefresh() now computes it fresh on every refresh instead of round-tripping through an MMKV key nothing ever wrote a real value into. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>VC-022</t>
+          <t>VC-020</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>A SendAck with seq 0 leaves the message permanently un-tickable and permanently duplicated</t>
+          <t>Concurrent applyServerMessages duplicates every row in the overlap, and can lose a whole batch on a conversation PK clash</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -18263,7 +18220,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-203</t>
+          <t>VC-UNIT-201</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
@@ -18274,24 +18231,24 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>normalizeSendAck has no test file at all. FIX: The outbox drain now rejects a SendAck with no usable seq (ack.seq is not &gt; 0) as a retryable server-kind AppError instead of writing it as a successful send — routes through the exact same retry path as any other transient send failure, so the row never gets stuck permanently un-tickable/duplicated. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>VC-001 makes this far more likely to be hit in practice, because seq gaps are constant. FIX: The three lookup queries in applyServerMessages moved inside db.write(), read before any prepareCreate/prepareUpdate call — closes the race without violating the prepare-then-batch-synchronously constraint. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>VC-026</t>
+          <t>VC-021</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Unread count climbs and the read watermark stalls for messages backfilled into the chat you are reading</t>
+          <t>applyReceipt is a non-atomic read-modify-write, so blue ticks can regress to grey</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -18301,7 +18258,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-207</t>
+          <t>VC-UNIT-202</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
@@ -18312,24 +18269,24 @@
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>VC-001 makes backfills constant, so this fires often. FIX: pageBackfill now mirrors the live-message path: if the backfilled page lands in the conversation on screen, it marks read (noteRead + clearUnread) instead of only noteDelivered. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>Every existing receipt test applies receipts sequentially, which is exactly why they all pass. FIX: applyReceipt now re-fetches the rows to update from inside db.write() (same pattern as VC-020) instead of before it, so the monotonic check is atomic with the write. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>VC-034</t>
+          <t>VC-022</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
+          <t>A SendAck with seq 0 leaves the message permanently un-tickable and permanently duplicated</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -18339,7 +18296,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-215</t>
+          <t>VC-UNIT-203</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -18350,24 +18307,24 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>normalizeSendAck has no test file at all. FIX: The outbox drain now rejects a SendAck with no usable seq (ack.seq is not &gt; 0) as a retryable server-kind AppError instead of writing it as a successful send — routes through the exact same retry path as any other transient send failure, so the row never gets stuck permanently un-tickable/duplicated. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>VC-035</t>
+          <t>VC-023</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>A misbuilt binary reports env:'dev' while talking to production</t>
+          <t>One 401 on send turns the entire outbox into permanently failed messages</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -18377,7 +18334,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-216</t>
+          <t>VC-UNIT-204</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -18388,19 +18345,19 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+          <t>FIX: classifySendFailure() grouped auth with client, treating a post-refresh-failure 401/403 as if THIS message were rejected (permanent:true, pauseDrain:false) — one transient auth hiccup then permanently failed every other queued message as the drain kept walking into the same 401. auth is a SESSION problem, not a message problem (client.ts already treats a refresh that cannot reach the server as retryable, leaving the session valid). Added a dedicated auth case returning {permanent:false, pauseDrain:true, cooldownMs:0}, matching the network/timeout/server treatment, so the drain pauses instead of destroying the queue and resumes once the session recovers. Split the existing it.each(['client','auth']) test (which encoded the old, wrong grouping) into client-only plus a new dedicated describe block for auth. Verified: full jest suite 452/452 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>VC-036</t>
+          <t>VC-024</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
+          <t>Migration-v3's five composite indexes never exist on a fresh install</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -18415,7 +18372,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>VC-UNIT-217</t>
+          <t>schema.test.ts: VC-024</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
@@ -18425,6 +18382,196 @@
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>FIX: added an unsafeSql hook to schema.ts (appSchema) — WatermelonDB's own supported extension point, confirmed by reading adapters/sqlite/encodeSchema/index.js (encodeSchema calls unsafeSql(sql, "setup") for a fresh install) — that appends the same five composite CREATE INDEX statements the v3 migration already applies on an upgrade. Extracted the five statements into a new shared compositeIndexes.ts so migrations.ts and schema.ts can never drift apart, and migrations.ts now maps over that same array instead of repeating the SQL inline. Verified: full jest suite 481/481 pass (3 new tests in schema.test.ts assert the hook exists, appends every composite index on kind:"setup", and leaves other DDL kinds untouched), tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>VC-026</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Unread count climbs and the read watermark stalls for messages backfilled into the chat you are reading</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-207</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>VC-001 makes backfills constant, so this fires often. FIX: pageBackfill now mirrors the live-message path: if the backfilled page lands in the conversation on screen, it marks read (noteRead + clearUnread) instead of only noteDelivered. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>VC-029</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Outbox backoff exhaustion is unreachable — MAX_SEND_ATTEMPTS can never fire</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-210</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>FIX: removed the dead attempt-count exhaustion path (MAX_SEND_ATTEMPTS/nextOutboxRetry in syncLogic.ts) that markFailed() fell back to only when permanent was omitted — a fallback no real call site ever triggered (SyncEngine.ts always passes a classified boolean from classifySendFailure()). This mechanism contradicted the documented WhatsApp-style policy (sendFailurePolicy.ts: reachability failures retry forever, never auto-fail by attempt count) and had no basis in the HLD/LLD spec (§L6 outbox semantics: classification-based retryable-vs-permanent only, no attempt cap). Made markFailed()'s permanent parameter required (compiler now prevents the dead path from ever coming back), updated the one test that accidentally relied on the old default (realtime-hardening.test.ts) to pass permanent explicitly, removed the 4 tests for the deleted dead function, and added a new regression test proving a retryable cause stays queued past a high attempt count. Verified: full jest suite 452/452 pass (455 - 4 removed + 1 added), tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>VC-034</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Retry-After is honored with an unbounded, uncancellable sleep</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-215</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>VC-035</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>A misbuilt binary reports env:'dev' while talking to production</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-216</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>VC-036</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Cold start after &gt;15 min idle opens the WebSocket with a certainly-expired token</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>dev branch, 2026-09-12</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>VC-UNIT-217</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Not independently tested</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>FIX: hasValidSession() added (tokens.ts); useAuthBootstrap now refreshes before hydrating on an expired-but-present token. hasSession() deliberately left presence-only to protect SyncEngine reconnect guards. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>

</xml_diff>

<commit_message>
feat(qa): mark VC-025/VC-027 fixed, log 6 production bugs to Tusha
Added VC-044 through VC-049 from manual production QA testing (contact
sync/display, presence delay, notification content/tap-through, and a
repeating email prompt), filed to Jira and assigned to Tusha Bhadouriya.

Added assignee support end to end: an optional assigneeAccountId on a
bug entry now sets the real Jira assignee field on create, and the
Excel Bugs sheet gained an Assignee column (appended at the end so no
existing column position shifts).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/QA/reports/VelChat-QA-Report.xlsx
+++ b/QA/reports/VelChat-QA-Report.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Results'!$A$4:$G$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bugs'!$A$1:$AA$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bugs'!$A$1:$AB$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Device Matrix'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Regression'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Flaky'!$A$1:$G$1</definedName>
@@ -629,7 +629,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-12 04:37 UTC</t>
+          <t>Generated 2026-09-12 05:00 UTC</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -11031,7 +11031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA44"/>
+  <dimension ref="A1:AB50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11061,6 +11061,7 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="44" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -11197,6 +11198,11 @@
       <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="AB1" s="4" t="inlineStr">
+        <is>
+          <t>Assignee</t>
         </is>
       </c>
     </row>
@@ -11343,6 +11349,7 @@
           <t>This one defect is the common cause behind VC-002, VC-003 and VC-004 — fix it first and re-test those before triaging them separately.</t>
         </is>
       </c>
+      <c r="AB2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -11483,6 +11490,7 @@
           <t>The client-side shape that triggers it: SyncEngine applies delivered then read for the same conversation with no gap.</t>
         </is>
       </c>
+      <c r="AB3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -11620,6 +11628,7 @@
         </is>
       </c>
       <c r="AA4" s="5" t="inlineStr"/>
+      <c r="AB4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -11755,6 +11764,7 @@
         </is>
       </c>
       <c r="AA5" s="5" t="inlineStr"/>
+      <c r="AB5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -11890,6 +11900,7 @@
         </is>
       </c>
       <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -12029,6 +12040,7 @@
           <t>DISCLOSURE: the QA harness uses this endpoint to provision its test identities, because it is currently the only way to obtain two real sessions without spending SMS. QA/lib/provision.js refuses to run against any non-local host unless QA_ALLOW_REMOTE_PROVISION=true. When this defect is fixed, switch the harness to OTP dev-mode (OTP_DEV_MODE=true) as documented in RUNBOOK.md.</t>
         </is>
       </c>
+      <c r="AB7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -12169,6 +12181,7 @@
           <t>Related client-side observation: warmBackend() (apps/mobile/src/infra/network/client.ts:33-62) pings the gateway, the gateway-proxied JWKS route and the realtime host. Because the gateway does not wake or reach its upstreams, that warm-up cannot actually warm identity/messaging/content/platform on Render. See VC-008.</t>
         </is>
       </c>
+      <c r="AB8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -12308,6 +12321,7 @@
           <t>Blocked on VC-007: if the gateway reached its upstreams, a proxied ping would wake them and this would resolve itself.</t>
         </is>
       </c>
+      <c r="AB9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -12446,6 +12460,7 @@
           <t>QA/lib/provision.js works around this by falling back to the identity-service origin, so downstream chat tests are not blocked. The workaround is documented in the file.</t>
         </is>
       </c>
+      <c r="AB10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -12584,6 +12599,7 @@
           <t>FIX: The request interceptor is now registered with {synchronous:true} (client.ts), so axios invokes it INLINE at the moment a request is issued instead of deferring it into a microtask. A call fired immediately before a synchronous clearSession() now reads the still-current token, closing the race. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -12724,6 +12740,7 @@
           <t>FIX: provision() now calls startPushRuntime() too (idempotent — harmless no-op on the normal first sign-in the App.tsx mount effect already started). A re-login after shutdownPushForSignOut() (sign-out) in the same process now correctly re-establishes the availability/message/session subscriptions instead of leaving them permanently torn down. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -12864,6 +12881,7 @@
           <t>FIX: refreshPermission() (pushService.ts) trusted hasNotificationPermission() alone, which on Android &lt;33 has no runtime dialog and unconditionally answers true regardless of the app-level or channel-level notification toggle the user can flip from system Settings. Combined it with the same native areMessageNotificationsBlocked() check the push blocker banner already used (getPushBlocker()), via a new pure decision function notificationsGranted(permitted, blocked) in pushState.ts, so permission now genuinely means the OS will show something on every API level before isPushAvailable lets the SyncEngine drop its background socket. No native code changed — reused the existing native primitive. Verified: full jest suite 456/456 pass (452 + 4 new), tsc --noEmit clean, eslint 0 errors on touched files. Could not be observed on a real Android &lt;=12 device (none available on this machine) — the fix is verified at the unit-test level against the exact documented defect (permitted=true, blocked=true -&gt; denied), not end-to-end on hardware.</t>
         </is>
       </c>
+      <c r="AB13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -13003,6 +13021,7 @@
           <t>FIX: sessionExpired() now runs the same purgeAccountData() as signOut() (extracted, shared), minus clearDeviceKey() (a transient expiry must still allow a later silent relogin) and the network logout call (pointless — the session is already rejected). The next sign-in on this device, even under a different phone number, no longer inherits the previous account chat DB, profile, contacts or receipts. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -13144,6 +13163,7 @@
           <t>FIX (investigated against the real backend source at D:Velchat, read-only): confirmed a refresh-reuse family revoke and a plain invalid/expired refresh both return an identical 401 UNAUTHORIZED with no distinguishing code, and confirmed device-key login is architecturally INDEPENDENT of the refresh-token family (revokeFamily only touches refresh_tokens; the devices table has no family_id) - so a device that still holds its private key can always mint a fresh session, and the client cannot and need not distinguish reuse-triggered revokes from ordinary rejections. Two real defects fixed: (1) clearSession() was deleting KVKeys.deviceId, which meant NEITHER the existing cold-start silent-relogin (useAuthBootstrap) NOR any warm recovery could ever actually reach /auth/challenge after a forced expiry, despite the code comments claiming this already worked - moved the explicit deviceId wipe into signOut() only, so a real logout is unchanged but a forced expiry now keeps it, same as the device key. (2) added attemptSilentRelogin() (authStore.ts), invoked from sessionExpired() itself, so a lost-refresh-response false-positive family revoke recovers IMMEDIATELY while the app is warm instead of only on the next cold start, turning a network hiccup back into nothing instead of stranding the user on the sign-in screen. Did not attempt to prevent the reuse-detection race itself (structurally requires a backend idempotency mechanism - out of scope, frontend-only per current instruction). Verified: full jest suite 481/481 pass, tsc --noEmit clean, eslint 0 errors. No RN-level test existed before; added 4 new tests (authStore.test.ts) covering the success, no-device-key, device-revoked and sessionExpired-wiring paths - the second and third caught the deviceId-wipe bug during RED before the fix was written.</t>
         </is>
       </c>
+      <c r="AB15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -13283,6 +13303,7 @@
           <t>FIX: Added cnfJktThumbprint() (deviceKey.ts) — a real RFC 7638 JWK thumbprint (RFC 8037 OKP encoding) over the device Ed25519 public key. doRefresh() now computes it fresh on every refresh instead of round-tripping through an MMKV key nothing ever wrote a real value into. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -13422,6 +13443,7 @@
           <t>Known and tracked as MP1 work, but it is the single highest-severity item in the client and should gate any release.</t>
         </is>
       </c>
+      <c r="AB17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -13561,6 +13583,7 @@
           <t>Needs an ADR or, at minimum, a scrub-on-cancel.</t>
         </is>
       </c>
+      <c r="AB18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -13699,6 +13722,7 @@
           <t>Grouped with VC-019: four of the five §A1/§D4 controls have no implementation.</t>
         </is>
       </c>
+      <c r="AB19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -13836,6 +13860,7 @@
           <t>Stated as coverage, not as a regression.</t>
         </is>
       </c>
+      <c r="AB20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -13975,6 +14000,7 @@
           <t>VC-001 makes this far more likely to be hit in practice, because seq gaps are constant. FIX: The three lookup queries in applyServerMessages moved inside db.write(), read before any prepareCreate/prepareUpdate call — closes the race without violating the prepare-then-batch-synchronously constraint. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -14113,6 +14139,7 @@
           <t>Every existing receipt test applies receipts sequentially, which is exactly why they all pass. FIX: applyReceipt now re-fetches the rows to update from inside db.write() (same pattern as VC-020) instead of before it, so the monotonic check is atomic with the write. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -14251,6 +14278,7 @@
           <t>normalizeSendAck has no test file at all. FIX: The outbox drain now rejects a SendAck with no usable seq (ack.seq is not &gt; 0) as a retryable server-kind AppError instead of writing it as a successful send — routes through the exact same retry path as any other transient send failure, so the row never gets stuck permanently un-tickable/duplicated. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -14390,6 +14418,7 @@
           <t>FIX: classifySendFailure() grouped auth with client, treating a post-refresh-failure 401/403 as if THIS message were rejected (permanent:true, pauseDrain:false) — one transient auth hiccup then permanently failed every other queued message as the drain kept walking into the same 401. auth is a SESSION problem, not a message problem (client.ts already treats a refresh that cannot reach the server as retryable, leaving the session valid). Added a dedicated auth case returning {permanent:false, pauseDrain:true, cooldownMs:0}, matching the network/timeout/server treatment, so the drain pauses instead of destroying the queue and resumes once the session recovers. Split the existing it.each(['client','auth']) test (which encoded the old, wrong grouping) into client-only plus a new dedicated describe block for auth. Verified: full jest suite 452/452 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -14528,6 +14557,7 @@
           <t>FIX: added an unsafeSql hook to schema.ts (appSchema) — WatermelonDB's own supported extension point, confirmed by reading adapters/sqlite/encodeSchema/index.js (encodeSchema calls unsafeSql(sql, "setup") for a fresh install) — that appends the same five composite CREATE INDEX statements the v3 migration already applies on an upgrade. Extracted the five statements into a new shared compositeIndexes.ts so migrations.ts and schema.ts can never drift apart, and migrations.ts now maps over that same array instead of repeating the SQL inline. Verified: full jest suite 481/481 pass (3 new tests in schema.test.ts assert the hook exists, appends every composite index on kind:"setup", and leaves other DDL kinds untouched), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -14663,6 +14693,7 @@
         </is>
       </c>
       <c r="AA26" s="5" t="inlineStr"/>
+      <c r="AB26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -14802,6 +14833,7 @@
           <t>VC-001 makes backfills constant, so this fires often. FIX: pageBackfill now mirrors the live-message path: if the backfilled page lands in the conversation on screen, it marks read (noteRead + clearUnread) instead of only noteDelivered. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -14936,6 +14968,7 @@
         </is>
       </c>
       <c r="AA28" s="5" t="inlineStr"/>
+      <c r="AB28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -15070,6 +15103,7 @@
         </is>
       </c>
       <c r="AA29" s="5" t="inlineStr"/>
+      <c r="AB29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -15208,6 +15242,7 @@
           <t>FIX: removed the dead attempt-count exhaustion path (MAX_SEND_ATTEMPTS/nextOutboxRetry in syncLogic.ts) that markFailed() fell back to only when permanent was omitted — a fallback no real call site ever triggered (SyncEngine.ts always passes a classified boolean from classifySendFailure()). This mechanism contradicted the documented WhatsApp-style policy (sendFailurePolicy.ts: reachability failures retry forever, never auto-fail by attempt count) and had no basis in the HLD/LLD spec (§L6 outbox semantics: classification-based retryable-vs-permanent only, no attempt cap). Made markFailed()'s permanent parameter required (compiler now prevents the dead path from ever coming back), updated the one test that accidentally relied on the old default (realtime-hardening.test.ts) to pass permanent explicitly, removed the 4 tests for the deleted dead function, and added a new regression test proving a retryable cause stays queued past a high attempt count. Verified: full jest suite 452/452 pass (455 - 4 removed + 1 added), tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -15343,6 +15378,7 @@
         </is>
       </c>
       <c r="AA31" s="5" t="inlineStr"/>
+      <c r="AB31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -15482,6 +15518,7 @@
           <t>The existing test passes only because sendText is invoked synchronously at the top of each handler — it cannot fail for the reason it claims.</t>
         </is>
       </c>
+      <c r="AB32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -15620,6 +15657,7 @@
           <t>The fix is one line: `if (seq &gt; 0 &amp;&amp; seq &lt;= store.lastSeq(conversationId)) return false`.</t>
         </is>
       </c>
+      <c r="AB33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -15759,6 +15797,7 @@
           <t>No JVM test source set exists — android/app/src contains only `main`. PushStore is plain-JVM-testable.</t>
         </is>
       </c>
+      <c r="AB34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -15897,6 +15936,7 @@
           <t>FIX: Retry-After is now clamped to [0, 10s] (MAX_RETRY_AFTER_MS, client.ts) before the wait, instead of obeying a server-supplied value unbounded. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -16035,6 +16075,7 @@
           <t>The prod URL fallback direction is defensible; make `name` fall back to 'prod' alongside it, or log.error when Config.API_BASE_URL is absent. FIX: Extracted the pure resolveAppEnv(rawName, rawApiBaseUrl, rawWsUrl) so the fallback logic is unit-testable. An unrecognised/missing ENV now falls back to 'prod' alongside the URL fallback (previously 'dev'), so a misbuilt binary can never report a safe-sounding name while actually pointing at production. Verified: full jest suite 455/455 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -16174,6 +16215,7 @@
           <t>FIX: hasValidSession() added (tokens.ts); useAuthBootstrap now refreshes before hydrating on an expired-but-present token. hasSession() deliberately left presence-only to protect SyncEngine reconnect guards. Verified: full jest suite 454/454 pass, tsc --noEmit clean, eslint 0 errors.</t>
         </is>
       </c>
+      <c r="AB37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -16312,6 +16354,7 @@
           <t>The one leak-into-logs path in the client itself is already mitigated by redact.ts's JWT pattern.</t>
         </is>
       </c>
+      <c r="AB38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -16446,6 +16489,7 @@
         </is>
       </c>
       <c r="AA39" s="5" t="inlineStr"/>
+      <c r="AB39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -16591,6 +16635,7 @@
           <t>Highest-impact finding of the run. It also leaves E2EE as the only remaining confidentiality control — and E2EE is not implemented yet (the client still sends plaintext `content`), so there is no compensating control today.</t>
         </is>
       </c>
+      <c r="AB40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -16729,6 +16774,7 @@
           <t>The same body-trusts-userId pattern appears in the notification prefs API and should be audited with it.</t>
         </is>
       </c>
+      <c r="AB41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
@@ -16866,6 +16912,7 @@
           <t>Fix together with VC-039.</t>
         </is>
       </c>
+      <c r="AB42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -17004,6 +17051,7 @@
           <t>The mobile composer disables send for empty input, so this is only reachable from a non-VelChat client — but it is still an unvalidated write.</t>
         </is>
       </c>
+      <c r="AB43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
@@ -17143,9 +17191,829 @@
           <t>Found during the 2026-09-11 re-verification pass (run verify-002), not in the original audit.</t>
         </is>
       </c>
+      <c r="AB44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>VC-044</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>VC-44</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Contact name/contact update does not sync immediately in chat UI</t>
+        </is>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Contact Sync / Contact Update</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>New Chat / Chat Screen / Contacts</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="O45" s="5" t="inlineStr">
+        <is>
+          <t>Unconfirmed — reported from manual production testing</t>
+        </is>
+      </c>
+      <c r="P45" s="5" t="inlineStr">
+        <is>
+          <t>A new contact is saved in the phone's contact list.</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>1. Save a new contact in the phone's address book.
+2. Open VelChat and enter that phone number / find the conversation.
+3. Observe only the phone number is shown, not the saved contact name.
+4. Send a message and exit the chat.
+5. Re-check — the contact name now appears, and multiple pending contact updates appear together instead of as they happen.</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>After saving the contact, VelChat should immediately detect/sync the contact and display the saved contact name consistently wherever that contact appears.</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>Initially only the phone number is displayed. After opening/chatting and then exiting the chat, the contact name appears. The contact information does not update immediately, and multiple contact-related updates appear together instead of updating immediately.</t>
+        </is>
+      </c>
+      <c r="T45" s="5" t="inlineStr">
+        <is>
+          <t>Users see raw phone numbers instead of contact names until they interact with the chat, which reads as broken contact sync.</t>
+        </is>
+      </c>
+      <c r="U45" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="V45" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated — reported from manual production QA testing, needs code-level triage.</t>
+        </is>
+      </c>
+      <c r="W45" s="5" t="inlineStr"/>
+      <c r="X45" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y45" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z45" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA45" s="5" t="inlineStr">
+        <is>
+          <t>Reported by Tusha Bhadouriya during production QA testing.</t>
+        </is>
+      </c>
+      <c r="AB45" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>VC-045</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>VC-45</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F46" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Real-Time Messaging / Notifications</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>Chat Screen / Notification</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>N/A — verification task</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P46" s="5" t="inlineStr">
+        <is>
+          <t>Two physical devices, each signed into a separate VelChat account.</t>
+        </is>
+      </c>
+      <c r="Q46" s="5" t="inlineStr">
+        <is>
+          <t>1. Exchange messages continuously between two devices for 10-13 minutes across different messaging scenarios via the normal Chat Page.
+2. Test notification-based replies from both devices for 6-8 minutes.
+3. Remove both apps from the background (swipe away / kill) and reply ONLY through notifications.
+4. Test a mixed scenario: one device replies through the notification while the other sends/replies normally from the Chat Page.</t>
+        </is>
+      </c>
+      <c r="R46" s="5" t="inlineStr">
+        <is>
+          <t>Messages and replies are delivered and synchronized correctly in real time across both devices in every tested scenario, including normal Chat Page messaging, notification replies, background-removed app state, and mixed notification + Chat Page messaging.</t>
+        </is>
+      </c>
+      <c r="S46" s="5" t="inlineStr">
+        <is>
+          <t>Not yet executed — result pending. Logged as a required verification pass across the scenarios above.</t>
+        </is>
+      </c>
+      <c r="T46" s="5" t="inlineStr">
+        <is>
+          <t>Any gap here directly breaks core messaging reliability and notification-reply delivery, the two most-used flows in the app.</t>
+        </is>
+      </c>
+      <c r="U46" s="5" t="inlineStr">
+        <is>
+          <t>N/A — this is a test-execution task, not yet a diagnosed defect.</t>
+        </is>
+      </c>
+      <c r="V46" s="5" t="inlineStr">
+        <is>
+          <t>N/A — pending test execution.</t>
+        </is>
+      </c>
+      <c r="W46" s="5" t="inlineStr"/>
+      <c r="X46" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y46" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z46" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA46" s="5" t="inlineStr">
+        <is>
+          <t>This entry tracks a two-device manual verification pass, not a confirmed defect. Assigned to Tusha Bhadouriya to execute and report actual pass/fail per scenario back into this bug.</t>
+        </is>
+      </c>
+      <c r="AB46" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>VC-046</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>VC-46</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Online/offline presence status updates with a noticeable delay</t>
+        </is>
+      </c>
+      <c r="E47" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Online/Offline Status</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Chat Screen / Contacts</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>Unconfirmed — reported from manual production testing</t>
+        </is>
+      </c>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>Two users in an active/visible chat.</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>1. Have the peer come online or go offline.
+2. Observe how long the status indicator takes to reflect the change.</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>When a user comes online or goes offline, their status should update and display immediately to other users.</t>
+        </is>
+      </c>
+      <c r="S47" s="5" t="inlineStr">
+        <is>
+          <t>The user's online/offline status is displayed after a noticeable delay.</t>
+        </is>
+      </c>
+      <c r="T47" s="5" t="inlineStr">
+        <is>
+          <t>Users see stale presence information, which can mislead them about whether the other person is actually available.</t>
+        </is>
+      </c>
+      <c r="U47" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated — could be a client-side polling/debounce delay or a backend presence-propagation delay.</t>
+        </is>
+      </c>
+      <c r="V47" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="W47" s="5" t="inlineStr"/>
+      <c r="X47" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y47" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z47" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA47" s="5" t="inlineStr">
+        <is>
+          <t>Reported by Tusha Bhadouriya during production QA testing. Root cause (client vs backend) not yet isolated.</t>
+        </is>
+      </c>
+      <c r="AB47" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>VC-047</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>VC-47</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Chat List shows the registered VelChat name instead of the saved contact name until a chat is opened</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Contact Name Sync</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Chat List / Message Yourself / Contact List</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M48" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="O48" s="5" t="inlineStr">
+        <is>
+          <t>Reported reproducible via Message Yourself</t>
+        </is>
+      </c>
+      <c r="P48" s="5" t="inlineStr">
+        <is>
+          <t>A contact is saved locally under a custom name different from their VelChat registered name (e.g. saved as "Aayush Sir" for an account registered as "Aayush Jain").</t>
+        </is>
+      </c>
+      <c r="Q48" s="5" t="inlineStr">
+        <is>
+          <t>1. Save a contact's number under a custom local name that differs from their VelChat display name.
+2. Open the Chat List — observe the registered VelChat name is shown instead of the saved contact name.
+3. Open the contact's chat via Message Yourself and return to the Chat List.
+4. Observe the name has now updated to the saved contact name.</t>
+        </is>
+      </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>The saved contact name should be displayed immediately in the Chat List wherever the contact is shown, without requiring the user to open the chat first.</t>
+        </is>
+      </c>
+      <c r="S48" s="5" t="inlineStr">
+        <is>
+          <t>Initially the registered VelChat name ("Aayush Jain") is displayed. After opening the contact's chat through Message Yourself and returning to the Chat List, it changes to the saved contact name ("Aayush Sir").</t>
+        </is>
+      </c>
+      <c r="T48" s="5" t="inlineStr">
+        <is>
+          <t>Users see the wrong display name for their own saved contacts until they happen to open that specific chat, which is confusing and looks like a sync bug.</t>
+        </is>
+      </c>
+      <c r="U48" s="5" t="inlineStr">
+        <is>
+          <t>Possibly the same underlying cause as the contact-sync bug reported separately — the Chat List may resolve the display name before local contact-name resolution/caching has run.</t>
+        </is>
+      </c>
+      <c r="V48" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="W48" s="5" t="inlineStr"/>
+      <c r="X48" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y48" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z48" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA48" s="5" t="inlineStr">
+        <is>
+          <t>Reported by Tusha Bhadouriya during production QA testing. May share a root cause with the contact-sync issue reported as a separate entry.</t>
+        </is>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>VC-048</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>VC-48</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Message notification omits the sender's name and tapping it does not open the chat</t>
+        </is>
+      </c>
+      <c r="E49" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Push Notifications / Notification Navigation</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Notification / Chat Screen</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr">
+        <is>
+          <t>Unconfirmed — reported from manual production testing</t>
+        </is>
+      </c>
+      <c r="P49" s="5" t="inlineStr">
+        <is>
+          <t>A message is received while the app is backgrounded.</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>1. Receive a new message while VelChat is backgrounded.
+2. Observe the notification only shows a generic count (e.g. "3 messages"), not who sent them.
+3. Tap the notification.
+4. Observe VelChat does not open directly — the user has to manually find and open the app from the app list.</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>The notification should display the sender's name along with the message/number of messages. Tapping the notification should directly open VelChat and navigate to the relevant chat.</t>
+        </is>
+      </c>
+      <c r="S49" s="5" t="inlineStr">
+        <is>
+          <t>The notification only shows VelChat and the number of messages, without identifying the sender. Tapping the notification does not open the app, requiring the user to manually open VelChat.</t>
+        </is>
+      </c>
+      <c r="T49" s="5" t="inlineStr">
+        <is>
+          <t>Users cannot tell who messaged them from the notification, and tapping it fails to take them to the conversation — a core notification-usability failure.</t>
+        </is>
+      </c>
+      <c r="U49" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated — possibly related to the existing duplicate-notification/pending-event defects already tracked in this registry, but not confirmed the same root cause.</t>
+        </is>
+      </c>
+      <c r="V49" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="W49" s="5" t="inlineStr"/>
+      <c r="X49" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y49" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z49" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA49" s="5" t="inlineStr">
+        <is>
+          <t>Reported by Tusha Bhadouriya during production QA testing.</t>
+        </is>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>VC-49</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>CLIENT</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Authentication / Profile / Email Verification</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Home Screen</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>Every login</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>Deterministic per report — every login</t>
+        </is>
+      </c>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>An account that already has an email address linked/saved.</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>1. Log in to an account that already has an email address associated with it.
+2. Observe the email-prompt bottom sheet on the Home Screen.</t>
+        </is>
+      </c>
+      <c r="R50" s="5" t="inlineStr">
+        <is>
+          <t>After logging in, the bottom sheet asking for an email should ONLY appear if the user has not added/linked an email. If the email is already present, the bottom sheet should not appear.</t>
+        </is>
+      </c>
+      <c r="S50" s="5" t="inlineStr">
+        <is>
+          <t>The bottom sheet asking for email opens repeatedly after every login, regardless of whether the user already has an email saved.</t>
+        </is>
+      </c>
+      <c r="T50" s="5" t="inlineStr">
+        <is>
+          <t>Users with an email already on file are repeatedly nagged for it on every login, a persistent, avoidable annoyance that looks like the app isn't remembering their profile.</t>
+        </is>
+      </c>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>The bottom-sheet trigger likely checks a stale/cached email-presence flag instead of current profile state, or the check itself is missing.</t>
+        </is>
+      </c>
+      <c r="V50" s="5" t="inlineStr">
+        <is>
+          <t>Not yet investigated.</t>
+        </is>
+      </c>
+      <c r="W50" s="5" t="inlineStr"/>
+      <c r="X50" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Y50" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="Z50" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA50" s="5" t="inlineStr">
+        <is>
+          <t>Reported by Tusha Bhadouriya during production QA testing.</t>
+        </is>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
+        <is>
+          <t>Tusha Bhadouriya</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1"/>
+  <autoFilter ref="A1:AB1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17156,7 +18024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -17309,7 +18177,7 @@
         </is>
       </c>
       <c r="B15" s="22" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C15" s="23" t="inlineStr"/>
     </row>
@@ -17320,7 +18188,7 @@
         </is>
       </c>
       <c r="B16" s="22" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C16" s="23" t="inlineStr"/>
     </row>
@@ -17342,7 +18210,7 @@
         </is>
       </c>
       <c r="B18" s="22" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C18" s="23" t="inlineStr"/>
     </row>
@@ -17412,7 +18280,7 @@
       </c>
       <c r="C26" s="25" t="inlineStr">
         <is>
-          <t>20 open P0/P1 defect(s) block the build.</t>
+          <t>22 open P0/P1 defect(s) block the build.</t>
         </is>
       </c>
     </row>
@@ -17762,6 +18630,40 @@
       <c r="C48" s="23" t="inlineStr">
         <is>
           <t>Concurrent refresh-token requests can all succeed — rotation is not race-safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>VC-045</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C49" s="23" t="inlineStr">
+        <is>
+          <t>Real-time messaging and notification-reply sync needs multi-scenario two-device verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>VC-049</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>Email-prompt bottom sheet reappears on every login even when an email is already saved</t>
         </is>
       </c>
     </row>

</xml_diff>